<commit_message>
Enforce structured addresses (BR-ADDR-002/003), stricter charset validation, update README
New rules: BR-ADDR-002 (Creditor address must be structured: StrtNm+TwnNm+Ctry),
BR-ADDR-003 (Debtor address consistency). SPS charset validation (BR-GEN-012)
now covers all text fields including remittance info and debtor address.

README updated with schema version table (SPS/EPC/CBPR+ all converge on
pain.001.001.09 by 2027), structured address requirements (Nov 2026),
roundtrip CLI docs, and updated rule counts (40+ rules, 13 violatable).

Test suite: 90 test cases, all Pass, all Round-Trip OK.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/testfaelle_comprehensive.xlsx
+++ b/templates/testfaelle_comprehensive.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S85"/>
+  <dimension ref="A1:S91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4850,6 +4850,306 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>TC-ADDR-001</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Strukturierte Adresse OK</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Vollstaendig strukturierte Creditor-Adresse</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>CH5604835012345678009</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>CHASUS33XXX</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>StrtNm, TwnNm, Ctry alle vorhanden</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>TC-ADDR-002</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Unvollstaendige Adresse</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>StrtNm fehlt in Creditor-Adresse</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>CH5604835012345678009</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>BARCGB22XXX</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>BR-ADDR-002</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>Violation entfernt StrtNm</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>TC-ADDR-003</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>SEPA strukturierte Adresse</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>SEPA mit vollstaendiger Adresse</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>CH5604835012345678009</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>SEPA mit strukturierter Adresse</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>TC-ADDR-004</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Domestic QR strukturierte Adresse</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>QR mit vollstaendiger Adresse</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Domestic-QR</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>CH5604835012345678009</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>1500</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>QR-Zahlung mit strukturierter Adresse</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>TC-CHAR-001</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>SPS-Zeichensatz OK</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Gueltige Zeichen im Creditor-Namen</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>CH5604835012345678009</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ABC Trading Co. (Int'l)</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>CHASUS33XXX</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>Alle Zeichen im SPS-Subset</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>TC-CHAR-002</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>SPS-Zeichensatz Sonderzeichen</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Erlaubte Sonderzeichen testen</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>SEPA</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>CH5604835012345678009</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Firma A/B - Test? Ja: (ok), +mehr</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>Alle erlaubten Sonderzeichen: / - ? : ( ) . , ' +</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Implement dual-standard support: SPS 2025 + CBPR+ SR2026
Per-testcase standard selection via new "Standard" Excel column
(sps2025 default, cbpr+2026 for SWIFT CBPR+).

Model changes:
- Standard enum (SPS_2025, CBPR_PLUS_2026) in testcase.py
- TestCase.standard field, AppConfig.cbpr_xsd_path

XSD validation:
- XsdValidator accepts dual schemas (SPS + CBPR+)
- Validates against correct schema per testcase standard
- Graceful error if CBPR+ XSD not configured

XML generation (CBPR+ mode):
- GrpHdr: NbOfTxs fixed "1", no CtrlSum
- PmtInf: no NbOfTxs, no CtrlSum
- PmtInfId = MsgId (CBPR+ Rule R8)
- CreDtTm with mandatory UTC offset
- UETR mandatory (already implemented)

8 new CBPR+ test cases (TC-CBPR-STD-001 to STD-NOK1) validated
against CBPR+ XSD. 112 total test cases, all passing.

Also: BR-REM-002 marked non-violatable (XSD maxLength=140 protects it),
.gitignore for docs/specs/cbpr+nonpublic/.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/testfaelle_comprehensive.xlsx
+++ b/templates/testfaelle_comprehensive.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S108"/>
+  <dimension ref="A1:T115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -544,6 +544,11 @@
           <t>Bemerkungen</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5583,27 +5588,27 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>TC-REM-NOK</t>
+          <t>TC-CB-JPY</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>SEPA Verwendungszweck zu lang</t>
+          <t>CBPR+ SAR nach Saudi-Arabien</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>SEPA mit Unstructured Remittance Info 141 Zeichen (ueber Maximum)</t>
+          <t>Cross-Border Zahlung in SAR mit Purpose-Code</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>SEPA</t>
+          <t>CBPR+</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -5622,53 +5627,68 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>800</v>
+        <v>50000</v>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>SAR</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Saudi Aramco Trading</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>SA0380000000608010167519</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>RIABORJX</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>Testtext fuer Remittance</t>
-        </is>
-      </c>
-      <c r="O98" t="inlineStr">
-        <is>
-          <t>BR-REM-002</t>
+          <t>Invoice INV-2026-JP-0044</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>CtgyPurp.Cd=SUPP; ChrgBr=SHAR</t>
         </is>
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>Erwartet: BR-REM-002 verletzt (USTRD &gt; 140 Zeichen)</t>
+          <t>SAR-Zahlung nach Saudi-Arabien (Japan hat kein IBAN)</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>TC-CB-JPY</t>
+          <t>TC-ADDR-006</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>CBPR+ SAR nach Saudi-Arabien</t>
+          <t>Domestic Creditor nur Country</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Cross-Border Zahlung in SAR mit Purpose-Code</t>
+          <t>Inlandszahlung CHF: Creditor-Adresse hat nur Country (NOK)</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>CBPR+</t>
+          <t>Domestic-IBAN</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -5687,68 +5707,48 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>50000</v>
+        <v>2200</v>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>SAR</t>
-        </is>
-      </c>
-      <c r="K99" t="inlineStr">
-        <is>
-          <t>Saudi Aramco Trading</t>
-        </is>
-      </c>
-      <c r="L99" t="inlineStr">
-        <is>
-          <t>SA0380000000608010167519</t>
-        </is>
-      </c>
-      <c r="M99" t="inlineStr">
-        <is>
-          <t>RIABORJX</t>
-        </is>
-      </c>
-      <c r="N99" t="inlineStr">
-        <is>
-          <t>Invoice INV-2026-JP-0044</t>
-        </is>
-      </c>
-      <c r="P99" t="inlineStr">
-        <is>
-          <t>CtgyPurp.Cd=SUPP; ChrgBr=SHAR</t>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>BR-ADDR-002</t>
         </is>
       </c>
       <c r="S99" t="inlineStr">
         <is>
-          <t>SAR-Zahlung nach Saudi-Arabien (Japan hat kein IBAN)</t>
+          <t>Erwartet: BR-ADDR-002 verletzt (StrtNm/TwnNm fehlt)</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>TC-ADDR-006</t>
+          <t>TC-CB-INVEST</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Domestic Creditor nur Country</t>
+          <t>CBPR+ AED Investment Dubai</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Inlandszahlung CHF: Creditor-Adresse hat nur Country (NOK)</t>
+          <t>Cross-Border Investmentzahlung nach UAE in AED</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Domestic-IBAN</t>
+          <t>CBPR+</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -5767,38 +5767,58 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>2200</v>
+        <v>75000</v>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>CHF</t>
-        </is>
-      </c>
-      <c r="O100" t="inlineStr">
-        <is>
-          <t>BR-ADDR-002</t>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Dubai Investment Fund LLC</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>AE070331234567890123456</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>ABORAEADXXX</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>Investment allocation Q1-2026 Ref IA-887</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>CtgyPurp.Cd=IVPT; ChrgBr=SHAR</t>
         </is>
       </c>
       <c r="S100" t="inlineStr">
         <is>
-          <t>Erwartet: BR-ADDR-002 verletzt (StrtNm/TwnNm fehlt)</t>
+          <t>Investment Purpose Code nach UAE</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>TC-CB-INVEST</t>
+          <t>TC-SEPA-BATCH</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>CBPR+ AED Investment Dubai</t>
+          <t>SEPA Batch 3 Transaktionen</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Cross-Border Investmentzahlung nach UAE in AED</t>
+          <t>SEPA mit 3 Creditors verschiedener Laender</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5808,7 +5828,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>CBPR+</t>
+          <t>SEPA</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -5827,87 +5847,37 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>75000</v>
+        <v>500</v>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>AED</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Dubai Investment Fund LLC</t>
+          <t>Berliner Handels GmbH</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>AE070331234567890123456</t>
-        </is>
-      </c>
-      <c r="M101" t="inlineStr">
-        <is>
-          <t>ABORAEADXXX</t>
+          <t>DE89370400440532013000</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>Investment allocation Q1-2026 Ref IA-887</t>
-        </is>
-      </c>
-      <c r="P101" t="inlineStr">
-        <is>
-          <t>CtgyPurp.Cd=IVPT; ChrgBr=SHAR</t>
+          <t>Rechnung RE-001</t>
         </is>
       </c>
       <c r="S101" t="inlineStr">
         <is>
-          <t>Investment Purpose Code nach UAE</t>
+          <t>Batch: 3 Transaktionen SEPA in verschiedene Laender</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>TC-SEPA-BATCH</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>SEPA Batch 3 Transaktionen</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>SEPA mit 3 Creditors verschiedener Laender</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>SEPA</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>Muster AG</t>
-        </is>
-      </c>
-      <c r="G102" t="inlineStr">
-        <is>
-          <t>CH5604835012345678009</t>
-        </is>
-      </c>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>CRESCHZZ80A</t>
-        </is>
-      </c>
       <c r="I102" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="J102" t="inlineStr">
         <is>
@@ -5916,28 +5886,23 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>Berliner Handels GmbH</t>
+          <t>Societe Parisienne SA</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>DE89370400440532013000</t>
+          <t>FR7630006000011234567890189</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>Rechnung RE-001</t>
-        </is>
-      </c>
-      <c r="S102" t="inlineStr">
-        <is>
-          <t>Batch: 3 Transaktionen SEPA in verschiedene Laender</t>
+          <t>Facture FA-002</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="I103" t="n">
-        <v>750</v>
+        <v>1200</v>
       </c>
       <c r="J103" t="inlineStr">
         <is>
@@ -5946,59 +5911,89 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Societe Parisienne SA</t>
+          <t>Banco di Roma SpA</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>FR7630006000011234567890189</t>
+          <t>IT60X0542811101000000123456</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>Facture FA-002</t>
+          <t>Fattura FT-003</t>
         </is>
       </c>
     </row>
     <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>TC-QR-EUR</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>QR-Zahlung EUR mit explizitem Creditor</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>QR-Zahlung in EUR mit manuell gesetztem Creditor</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Domestic-QR</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Muster AG</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>CH5604835012345678009</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>CRESCHZZ80A</t>
+        </is>
+      </c>
       <c r="I104" t="n">
-        <v>1200</v>
+        <v>890</v>
       </c>
       <c r="J104" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="K104" t="inlineStr">
-        <is>
-          <t>Banco di Roma SpA</t>
-        </is>
-      </c>
-      <c r="L104" t="inlineStr">
-        <is>
-          <t>IT60X0542811101000000123456</t>
-        </is>
-      </c>
-      <c r="N104" t="inlineStr">
-        <is>
-          <t>Fattura FT-003</t>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>QR-IBAN mit EUR statt CHF (beides erlaubt)</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>TC-QR-EUR</t>
+          <t>TC-CB-MULTI1</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>QR-Zahlung EUR mit explizitem Creditor</t>
+          <t>CBPR+ Multi-Currency Gruppe 1</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>QR-Zahlung in EUR mit manuell gesetztem Creditor</t>
+          <t>Multi-Payment: CBPR+ USD und GBP in einer XML</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -6008,7 +6003,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Domestic-QR</t>
+          <t>CBPR+</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -6027,33 +6022,48 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>890</v>
+        <v>20000</v>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>CHASUS33</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>Wire transfer March 2026</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>GroupId=BATCH-CBPR</t>
         </is>
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>QR-IBAN mit EUR statt CHF (beides erlaubt)</t>
+          <t>Gruppe BATCH-CBPR: PmtInf 1 (USD)</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>TC-CB-MULTI1</t>
+          <t>TC-CB-MULTI2</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>CBPR+ Multi-Currency Gruppe 1</t>
+          <t>CBPR+ Multi-Currency Gruppe 2</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Multi-Payment: CBPR+ USD und GBP in einer XML</t>
+          <t>Multi-Payment: CBPR+ GBP Teil</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6082,48 +6092,48 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>20000</v>
+        <v>15000</v>
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>CHASUS33</t>
+          <t>BARCGB22</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t>Wire transfer March 2026</t>
+          <t>Payment ref GBP-2026-03</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>GroupId=BATCH-CBPR</t>
+          <t>GroupId=BATCH-CBPR; ChrgBr=DEBT</t>
         </is>
       </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t>Gruppe BATCH-CBPR: PmtInf 1 (USD)</t>
+          <t>Gruppe BATCH-CBPR: PmtInf 2 (GBP)</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>TC-CB-MULTI2</t>
+          <t>TC-IBAN-MAX</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>CBPR+ Multi-Currency Gruppe 2</t>
+          <t>Domestic-IBAN Grossbetrag mit SCOR</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Multi-Payment: CBPR+ GBP Teil</t>
+          <t>Hoher CHF-Betrag mit SCOR-Referenz und vollem Debtor</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6133,12 +6143,12 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>CBPR+</t>
+          <t>Domestic-IBAN</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Muster AG</t>
+          <t>Schweizerische Nationalbank</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -6148,52 +6158,42 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>CRESCHZZ80A</t>
+          <t>SNBZCHZZXXX</t>
         </is>
       </c>
       <c r="I107" t="n">
-        <v>15000</v>
+        <v>5000000</v>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="M107" t="inlineStr">
-        <is>
-          <t>BARCGB22</t>
-        </is>
-      </c>
-      <c r="N107" t="inlineStr">
-        <is>
-          <t>Payment ref GBP-2026-03</t>
-        </is>
-      </c>
-      <c r="P107" t="inlineStr">
-        <is>
-          <t>GroupId=BATCH-CBPR; ChrgBr=DEBT</t>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Kantonsspital Zuerich</t>
         </is>
       </c>
       <c r="S107" t="inlineStr">
         <is>
-          <t>Gruppe BATCH-CBPR: PmtInf 2 (GBP)</t>
+          <t>5 Mio CHF Inlandszahlung mit BIC 11 Stellen</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>TC-IBAN-MAX</t>
+          <t>TC-CBPR-STD-001</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Domestic-IBAN Grossbetrag mit SCOR</t>
+          <t>CBPR+ Standard USD-Zahlung</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Hoher CHF-Betrag mit SCOR-Referenz und vollem Debtor</t>
+          <t>CBPR+ XSD: einfache USD-Zahlung nach USA</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6203,12 +6203,12 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Domestic-IBAN</t>
+          <t>CBPR+</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Schweizerische Nationalbank</t>
+          <t>Muster AG</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -6218,25 +6218,630 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>SNBZCHZZXXX</t>
+          <t>CRESCHZZ80A</t>
         </is>
       </c>
       <c r="I108" t="n">
-        <v>5000000</v>
+        <v>10000</v>
       </c>
       <c r="J108" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Acme International SA</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>FR7630006000011234567890189</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>BNPAFRPP</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>Invoice INV-2026-001</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>ChrgBr=SHAR</t>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>CBPR+ USD via FR IBAN (USA hat kein IBAN)</t>
+        </is>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>cbpr+2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>TC-CBPR-STD-002</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>CBPR+ Standard GBP-Zahlung</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>CBPR+ XSD: GBP-Zahlung nach UK</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Muster AG</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>CH5604835012345678009</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>CRESCHZZ80A</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>British Trading Ltd</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>GB29NWBK60161331926819</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>NWBKGB2L</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>Payment March 2026</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>ChrgBr=DEBT</t>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>CBPR+ GBP mit DEBT</t>
+        </is>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>cbpr+2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>TC-CBPR-STD-003</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>CBPR+ Standard EUR-Zahlung</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>CBPR+ XSD: EUR-Zahlung nach Deutschland</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Muster AG</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>CH5604835012345678009</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>CRESCHZZ80A</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Deutsche Bank AG</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>DE89370400440532013000</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>DEUTDEFF</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>Contract payment</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>ChrgBr=CRED</t>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>CBPR+ EUR mit CRED</t>
+        </is>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>cbpr+2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>TC-CBPR-STD-004</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>CBPR+ CHF nach Saudi-Arabien</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>CBPR+ XSD: CHF-Zahlung mit Purpose-Code</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Muster AG</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>CH5604835012345678009</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>CRESCHZZ80A</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>50000</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr">
-        <is>
-          <t>Kantonsspital Zuerich</t>
-        </is>
-      </c>
-      <c r="S108" t="inlineStr">
-        <is>
-          <t>5 Mio CHF Inlandszahlung mit BIC 11 Stellen</t>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Saudi Aramco Trading</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>SA0380000000608010167519</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>RIABORJX</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>Oil supply Q1-2026</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>ChrgBr=SHAR; CtgyPurp.Cd=SUPP</t>
+        </is>
+      </c>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>CBPR+ CHF mit Purpose SUPP</t>
+        </is>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>cbpr+2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>TC-CBPR-STD-005</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>CBPR+ Maximal optionale Felder</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>CBPR+ XSD: alle optionalen Felder genutzt</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Muster AG</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>CH5604835012345678009</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>CRESCHZZ80A</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Globex International</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>GB82WEST12345698765432</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>WESTGB2L</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>Final settlement REF-44891</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>ChrgBr=DEBT; CtgyPurp.Cd=SUPP; PmtId.InstrId=INSTR-CBPR-001; UltmtDbtr.Nm=Muster Holding AG; UltmtDbtr.PstlAdr.TwnNm=Zug; UltmtDbtr.PstlAdr.Ctry=CH; UltmtCdtr.Nm=Globex Corp; UltmtCdtr.PstlAdr.TwnNm=London; UltmtCdtr.PstlAdr.Ctry=GB</t>
+        </is>
+      </c>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>CBPR+ XSD mit UltmtDbtr, UltmtCdtr, InstrId, CtgyPurp</t>
+        </is>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>cbpr+2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>TC-CBPR-STD-006</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>CBPR+ AED Investment</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>CBPR+ XSD: AED-Zahlung nach UAE</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Muster AG</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>CH5604835012345678009</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>CRESCHZZ80A</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>75000</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Emirates Investment Fund</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>AE070331234567890123456</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>ABORAEADXXX</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>Investment Q1-2026</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>ChrgBr=SHAR; CtgyPurp.Cd=IVPT</t>
+        </is>
+      </c>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>CBPR+ AED nach UAE</t>
+        </is>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>cbpr+2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>TC-CBPR-STD-007</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>CBPR+ Gehaltszahlung</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>CBPR+ XSD: Gehaltszahlung mit SALA Purpose</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Muster AG</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>CH5604835012345678009</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>CRESCHZZ80A</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>8500</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>John Smith</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>GB29NWBK60161331926819</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>NWBKGB2L</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>Salary March 2026</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>ChrgBr=DEBT; CtgyPurp.Cd=SALA</t>
+        </is>
+      </c>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t>CBPR+ Gehaltszahlung</t>
+        </is>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>cbpr+2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>TC-CBPR-STD-NOK1</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>CBPR+ mit SLEV verboten</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>CBPR+ XSD: SLEV als ChrgBr nicht erlaubt</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Muster AG</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>CH5604835012345678009</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>CRESCHZZ80A</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>CHASUS33</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>BR-CBPR-003</t>
+        </is>
+      </c>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t>CBPR+ verbietet SLEV</t>
+        </is>
+      </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>cbpr+2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add sps2025 standard to all SPS test cases, regenerate all examples
- Set Standard=sps2025 on all 104 SPS test cases (was empty/default)
- Set Standard=cbpr+2026 on all 8 CBPR+ test cases (unchanged)
- Regenerate all 111 XML example files (103 SPS + 8 CBPR+)
- Independent re-validation: all 111 XMLs pass their respective XSD

112 test cases total (104 SPS + 8 CBPR+), 0 Fail.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/testfaelle_comprehensive.xlsx
+++ b/templates/testfaelle_comprehensive.xlsx
@@ -594,6 +594,11 @@
           <t>Basis-SEPA</t>
         </is>
       </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -639,6 +644,11 @@
           <t>BR-SEPA-001</t>
         </is>
       </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -684,6 +694,11 @@
           <t>BR-SEPA-003</t>
         </is>
       </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -729,6 +744,11 @@
           <t>BR-SEPA-004</t>
         </is>
       </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -769,6 +789,11 @@
           <t>CHF</t>
         </is>
       </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -814,6 +839,11 @@
           <t>BR-QR-002</t>
         </is>
       </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -859,6 +889,11 @@
           <t>BR-QR-003</t>
         </is>
       </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -904,6 +939,11 @@
           <t>BR-QR-004</t>
         </is>
       </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -944,6 +984,11 @@
           <t>CHF</t>
         </is>
       </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -989,6 +1034,11 @@
           <t>BR-IBAN-001</t>
         </is>
       </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1034,6 +1084,11 @@
           <t>BR-IBAN-002</t>
         </is>
       </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1079,6 +1134,11 @@
           <t>BR-IBAN-004</t>
         </is>
       </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1134,6 +1194,11 @@
           <t>Charge Bearer DEBT</t>
         </is>
       </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1189,6 +1254,11 @@
           <t>Charge Bearer CRED</t>
         </is>
       </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1244,6 +1314,11 @@
           <t>Charge Bearer SHAR</t>
         </is>
       </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1304,6 +1379,11 @@
           <t>Violation setzt ChrgBr auf INVALID</t>
         </is>
       </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1354,6 +1434,11 @@
           <t>BR-CBPR-005</t>
         </is>
       </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1409,6 +1494,11 @@
           <t>Unstrukturierte Remittance Info</t>
         </is>
       </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1464,6 +1554,11 @@
           <t>Grenzwert-Test: genau 140 Zeichen</t>
         </is>
       </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1514,6 +1609,11 @@
           <t>Exotische aber gueltige Waehrung</t>
         </is>
       </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1564,6 +1664,11 @@
           <t>Waehrung USD, Land US</t>
         </is>
       </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1614,6 +1719,11 @@
           <t>Waehrung JPY, Land JP</t>
         </is>
       </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1664,6 +1774,11 @@
           <t>Waehrung GBP, Land GB</t>
         </is>
       </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1714,6 +1829,11 @@
           <t>Waehrung CNY, Land CN</t>
         </is>
       </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1764,6 +1884,11 @@
           <t>Waehrung AUD, Land AU</t>
         </is>
       </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1814,6 +1939,11 @@
           <t>Waehrung CAD, Land CA</t>
         </is>
       </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1864,6 +1994,11 @@
           <t>Waehrung HKD, Land HK</t>
         </is>
       </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1914,6 +2049,11 @@
           <t>Waehrung SGD, Land SG</t>
         </is>
       </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1964,6 +2104,11 @@
           <t>Waehrung SEK, Land SE</t>
         </is>
       </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2014,6 +2159,11 @@
           <t>Waehrung KRW, Land KR</t>
         </is>
       </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2064,6 +2214,11 @@
           <t>Waehrung NOK, Land NO</t>
         </is>
       </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2114,6 +2269,11 @@
           <t>Waehrung NZD, Land AU</t>
         </is>
       </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2164,6 +2324,11 @@
           <t>Waehrung INR, Land IN</t>
         </is>
       </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2214,6 +2379,11 @@
           <t>Waehrung MXN, Land MX</t>
         </is>
       </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2264,6 +2434,11 @@
           <t>Waehrung TWD, Land HK</t>
         </is>
       </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2314,6 +2489,11 @@
           <t>Waehrung ZAR, Land ZA</t>
         </is>
       </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2364,6 +2544,11 @@
           <t>Waehrung BRL, Land BR</t>
         </is>
       </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2414,6 +2599,11 @@
           <t>Waehrung DKK, Land DK</t>
         </is>
       </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2464,6 +2654,11 @@
           <t>Waehrung PLN, Land PL</t>
         </is>
       </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2514,6 +2709,11 @@
           <t>Waehrung THB, Land TH</t>
         </is>
       </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2564,6 +2764,11 @@
           <t>Waehrung ILS, Land IL</t>
         </is>
       </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2614,6 +2819,11 @@
           <t>Waehrung IDR, Land SG</t>
         </is>
       </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2664,6 +2874,11 @@
           <t>Waehrung CZK, Land CZ</t>
         </is>
       </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2714,6 +2929,11 @@
           <t>Waehrung AED, Land AE</t>
         </is>
       </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2764,6 +2984,11 @@
           <t>Waehrung TRY, Land TR</t>
         </is>
       </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2814,6 +3039,11 @@
           <t>Waehrung HUF, Land HU</t>
         </is>
       </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2864,6 +3094,11 @@
           <t>Waehrung SAR, Land SA</t>
         </is>
       </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2914,6 +3149,11 @@
           <t>Waehrung PHP, Land SG</t>
         </is>
       </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2969,6 +3209,11 @@
           <t>Agent wird entfernt fuer USD</t>
         </is>
       </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3024,6 +3269,11 @@
           <t>Agent wird entfernt fuer JPY</t>
         </is>
       </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3079,6 +3329,11 @@
           <t>Agent wird entfernt fuer GBP</t>
         </is>
       </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3134,6 +3389,11 @@
           <t>Agent wird entfernt fuer CNY</t>
         </is>
       </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3189,6 +3449,11 @@
           <t>Agent wird entfernt fuer AUD</t>
         </is>
       </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3244,6 +3509,11 @@
           <t>Agent wird entfernt fuer CAD</t>
         </is>
       </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3299,6 +3569,11 @@
           <t>Agent wird entfernt fuer HKD</t>
         </is>
       </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3354,6 +3629,11 @@
           <t>Agent wird entfernt fuer SGD</t>
         </is>
       </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3409,6 +3689,11 @@
           <t>Agent wird entfernt fuer SEK</t>
         </is>
       </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3464,6 +3749,11 @@
           <t>Agent wird entfernt fuer KRW</t>
         </is>
       </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3519,6 +3809,11 @@
           <t>Agent wird entfernt fuer NOK</t>
         </is>
       </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3574,6 +3869,11 @@
           <t>Agent wird entfernt fuer NZD</t>
         </is>
       </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3629,6 +3929,11 @@
           <t>Agent wird entfernt fuer INR</t>
         </is>
       </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3684,6 +3989,11 @@
           <t>Agent wird entfernt fuer MXN</t>
         </is>
       </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3739,6 +4049,11 @@
           <t>Agent wird entfernt fuer TWD</t>
         </is>
       </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3794,6 +4109,11 @@
           <t>Agent wird entfernt fuer ZAR</t>
         </is>
       </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3849,6 +4169,11 @@
           <t>Agent wird entfernt fuer BRL</t>
         </is>
       </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3904,6 +4229,11 @@
           <t>Agent wird entfernt fuer DKK</t>
         </is>
       </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3959,6 +4289,11 @@
           <t>Agent wird entfernt fuer PLN</t>
         </is>
       </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4014,6 +4349,11 @@
           <t>Agent wird entfernt fuer THB</t>
         </is>
       </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4069,6 +4409,11 @@
           <t>Agent wird entfernt fuer ILS</t>
         </is>
       </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4124,6 +4469,11 @@
           <t>Agent wird entfernt fuer IDR</t>
         </is>
       </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4179,6 +4529,11 @@
           <t>Agent wird entfernt fuer CZK</t>
         </is>
       </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4234,6 +4589,11 @@
           <t>Agent wird entfernt fuer AED</t>
         </is>
       </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4289,6 +4649,11 @@
           <t>Agent wird entfernt fuer TRY</t>
         </is>
       </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4344,6 +4709,11 @@
           <t>Agent wird entfernt fuer HUF</t>
         </is>
       </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4399,6 +4769,11 @@
           <t>Agent wird entfernt fuer SAR</t>
         </is>
       </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4454,6 +4829,11 @@
           <t>Agent wird entfernt fuer PHP</t>
         </is>
       </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4504,6 +4884,11 @@
           <t>SEPA-Land DE mit Nicht-EUR Waehrung</t>
         </is>
       </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4554,6 +4939,11 @@
           <t>SEPA-Land FR mit Nicht-EUR Waehrung</t>
         </is>
       </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4604,6 +4994,11 @@
           <t>SEPA-Land IT mit Nicht-EUR Waehrung</t>
         </is>
       </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4654,6 +5049,11 @@
           <t>SEPA-Land ES mit Nicht-EUR Waehrung</t>
         </is>
       </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4704,6 +5104,11 @@
           <t>SEPA-Land NL mit Nicht-EUR Waehrung</t>
         </is>
       </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4754,6 +5159,11 @@
           <t>SEPA-Land BE mit Nicht-EUR Waehrung</t>
         </is>
       </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4804,6 +5214,11 @@
           <t>SEPA-Land AT mit Nicht-EUR Waehrung</t>
         </is>
       </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4854,6 +5269,11 @@
           <t>SEPA-Land PT mit Nicht-EUR Waehrung</t>
         </is>
       </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4904,6 +5324,11 @@
           <t>StrtNm, TwnNm, Ctry alle vorhanden</t>
         </is>
       </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4959,6 +5384,11 @@
           <t>Violation entfernt StrtNm</t>
         </is>
       </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -5004,6 +5434,11 @@
           <t>SEPA mit strukturierter Adresse</t>
         </is>
       </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5049,6 +5484,11 @@
           <t>QR-Zahlung mit strukturierter Adresse</t>
         </is>
       </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5104,6 +5544,11 @@
           <t>Alle Zeichen im SPS-Subset</t>
         </is>
       </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5154,6 +5599,11 @@
           <t>Alle erlaubten Sonderzeichen: / - ? : ( ) . , ' +</t>
         </is>
       </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5214,6 +5664,11 @@
           <t>Erwartet: BR-ADDR-002 verletzt (strukturierte Adresse fehlt)</t>
         </is>
       </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5294,6 +5749,11 @@
           <t>CBPR+ CHF ueber UAE IBAN mit Purpose-Code TAXS</t>
         </is>
       </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5374,6 +5834,11 @@
           <t>Alle optionalen B/C-Level Felder genutzt: UltmtDbtr, UltmtCdtr, InstrId, CtgyPurp, BtchBookg, ChrgBr=DEBT</t>
         </is>
       </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5444,6 +5909,11 @@
           <t>Erwartet: BR-CBPR-003 verletzt (SLEV bei CBPR+ verboten)</t>
         </is>
       </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5524,6 +5994,11 @@
           <t>Gehaltszahlung mit Purpose-Code</t>
         </is>
       </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5584,6 +6059,11 @@
           <t>Grenzwert: exakt 140 Zeichen Verwendungszweck</t>
         </is>
       </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5664,6 +6144,11 @@
           <t>SAR-Zahlung nach Saudi-Arabien (Japan hat kein IBAN)</t>
         </is>
       </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5724,6 +6209,11 @@
           <t>Erwartet: BR-ADDR-002 verletzt (StrtNm/TwnNm fehlt)</t>
         </is>
       </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5804,6 +6294,11 @@
           <t>Investment Purpose Code nach UAE</t>
         </is>
       </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5872,6 +6367,11 @@
       <c r="S101" t="inlineStr">
         <is>
           <t>Batch: 3 Transaktionen SEPA in verschiedene Laender</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>sps2025</t>
         </is>
       </c>
     </row>
@@ -5979,6 +6479,11 @@
           <t>QR-IBAN mit EUR statt CHF (beides erlaubt)</t>
         </is>
       </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -6049,6 +6554,11 @@
           <t>Gruppe BATCH-CBPR: PmtInf 1 (USD)</t>
         </is>
       </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -6119,6 +6629,11 @@
           <t>Gruppe BATCH-CBPR: PmtInf 2 (GBP)</t>
         </is>
       </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>sps2025</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -6177,6 +6692,11 @@
       <c r="S107" t="inlineStr">
         <is>
           <t>5 Mio CHF Inlandszahlung mit BIC 11 Stellen</t>
+        </is>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>sps2025</t>
         </is>
       </c>
     </row>

</xml_diff>